<commit_message>
Update users.xlsx seed data: Modify user data in the Excel file to reflect recent changes and improvements for testing and development purposes.
</commit_message>
<xml_diff>
--- a/popy-be/seed-data/users.xlsx
+++ b/popy-be/seed-data/users.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>email</t>
   </si>
@@ -142,13 +142,19 @@
   </si>
   <si>
     <t>Ruwan Bandara</t>
+  </si>
+  <si>
+    <t>popy@gmail.com</t>
+  </si>
+  <si>
+    <t>Sks732^%@</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,6 +167,20 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Lucida Console"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -205,10 +225,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -219,8 +240,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -521,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -765,8 +789,20 @@
         <v>21</v>
       </c>
     </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H9"/>
+  <hyperlinks>
+    <hyperlink ref="B11" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>